<commit_message>
first semifinals leg acb 2025-2026
</commit_message>
<xml_diff>
--- a/informes_data/ACB/2025-26/playoffs/aggregate_individual/AGG_IND_Barça.xlsx
+++ b/informes_data/ACB/2025-26/playoffs/aggregate_individual/AGG_IND_Barça.xlsx
@@ -562,76 +562,76 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D2" t="n">
-        <v>24.4467</v>
+        <v>33.7133</v>
       </c>
       <c r="E2" t="n">
-        <v>6.2127</v>
+        <v>12.9768</v>
       </c>
       <c r="F2" t="n">
-        <v>18.234</v>
+        <v>20.7364</v>
       </c>
       <c r="G2" t="n">
-        <v>24.8643</v>
+        <v>30.2633</v>
       </c>
       <c r="H2" t="n">
-        <v>15.648</v>
+        <v>19.8114</v>
       </c>
       <c r="I2" t="n">
-        <v>9.2166</v>
+        <v>10.4519</v>
       </c>
       <c r="J2" t="n">
-        <v>20.7645</v>
+        <v>25.0465</v>
       </c>
       <c r="K2" t="n">
-        <v>17.2272</v>
+        <v>20.3654</v>
       </c>
       <c r="L2" t="n">
-        <v>3.5376</v>
+        <v>4.6811</v>
       </c>
       <c r="M2" t="n">
-        <v>4.0998</v>
+        <v>5.2166</v>
       </c>
       <c r="N2" t="n">
-        <v>-1.5789</v>
+        <v>-0.5542999999999999</v>
       </c>
       <c r="O2" t="n">
-        <v>5.678999999999999</v>
+        <v>5.7709</v>
       </c>
       <c r="P2" t="n">
-        <v>-6.2307</v>
+        <v>-3.4975</v>
       </c>
       <c r="Q2" t="n">
-        <v>-17.3064</v>
+        <v>-17.4876</v>
       </c>
       <c r="R2" t="n">
-        <v>11.0763</v>
+        <v>13.9901</v>
       </c>
       <c r="S2" t="n">
-        <v>0.9663</v>
+        <v>2.1447</v>
       </c>
       <c r="T2" t="n">
-        <v>-2.5305</v>
+        <v>-1.3979</v>
       </c>
       <c r="U2" t="n">
-        <v>3.4962</v>
+        <v>3.5426</v>
       </c>
       <c r="V2" t="n">
-        <v>4.8465</v>
+        <v>4.803</v>
       </c>
       <c r="W2" t="n">
-        <v>5.2851</v>
+        <v>6.8156</v>
       </c>
       <c r="X2" t="n">
-        <v>-0.4386</v>
+        <v>-2.0129</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>W. CLYBURN</t>
+          <t>N. LAPROVITTOLA</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -640,76 +640,76 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D3" t="n">
-        <v>21.1923</v>
+        <v>25.3924</v>
       </c>
       <c r="E3" t="n">
-        <v>14.8923</v>
+        <v>19.7664</v>
       </c>
       <c r="F3" t="n">
-        <v>6.300000000000001</v>
+        <v>5.625599999999999</v>
       </c>
       <c r="G3" t="n">
-        <v>20.6316</v>
+        <v>25.4082</v>
       </c>
       <c r="H3" t="n">
-        <v>0.6026999999999987</v>
+        <v>4.1893</v>
       </c>
       <c r="I3" t="n">
-        <v>20.0289</v>
+        <v>21.2189</v>
       </c>
       <c r="J3" t="n">
-        <v>22.6773</v>
+        <v>24.0299</v>
       </c>
       <c r="K3" t="n">
-        <v>-0.3245999999999998</v>
+        <v>2.8042</v>
       </c>
       <c r="L3" t="n">
-        <v>23.0016</v>
+        <v>21.2257</v>
       </c>
       <c r="M3" t="n">
-        <v>-2.0451</v>
+        <v>1.3783</v>
       </c>
       <c r="N3" t="n">
-        <v>0.9273000000000002</v>
+        <v>1.3852</v>
       </c>
       <c r="O3" t="n">
-        <v>-2.9727</v>
+        <v>-0.006800000000000028</v>
       </c>
       <c r="P3" t="n">
-        <v>-1.3848</v>
+        <v>-5.3626</v>
       </c>
       <c r="Q3" t="n">
-        <v>-15.9222</v>
+        <v>-10.2593</v>
       </c>
       <c r="R3" t="n">
-        <v>14.5374</v>
+        <v>4.8964</v>
       </c>
       <c r="S3" t="n">
-        <v>4.737299999999999</v>
+        <v>2.1449</v>
       </c>
       <c r="T3" t="n">
-        <v>-0.8175</v>
+        <v>0.6594</v>
       </c>
       <c r="U3" t="n">
-        <v>5.5548</v>
+        <v>1.4856</v>
       </c>
       <c r="V3" t="n">
-        <v>-2.7921</v>
+        <v>3.2019</v>
       </c>
       <c r="W3" t="n">
-        <v>8.954699999999999</v>
+        <v>5.3366</v>
       </c>
       <c r="X3" t="n">
-        <v>-11.7471</v>
+        <v>-2.1346</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>N. LAPROVITTOLA</t>
+          <t>J. VESELY</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -718,70 +718,70 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="D4" t="n">
-        <v>18.8871</v>
+        <v>24.424</v>
       </c>
       <c r="E4" t="n">
-        <v>13.2633</v>
+        <v>13.6752</v>
       </c>
       <c r="F4" t="n">
-        <v>5.6238</v>
+        <v>10.7488</v>
       </c>
       <c r="G4" t="n">
-        <v>14.9715</v>
+        <v>3.0991</v>
       </c>
       <c r="H4" t="n">
-        <v>3.4887</v>
+        <v>3.523000000000001</v>
       </c>
       <c r="I4" t="n">
-        <v>11.4825</v>
+        <v>-0.4235000000000002</v>
       </c>
       <c r="J4" t="n">
-        <v>14.3661</v>
+        <v>5.273999999999999</v>
       </c>
       <c r="K4" t="n">
-        <v>2.9958</v>
+        <v>3.212</v>
       </c>
       <c r="L4" t="n">
-        <v>11.3703</v>
+        <v>2.0621</v>
       </c>
       <c r="M4" t="n">
-        <v>0.6051</v>
+        <v>-2.1749</v>
       </c>
       <c r="N4" t="n">
-        <v>0.4929</v>
+        <v>0.3107000000000002</v>
       </c>
       <c r="O4" t="n">
-        <v>0.1122</v>
+        <v>-2.4854</v>
       </c>
       <c r="P4" t="n">
-        <v>-0.6923999999999997</v>
+        <v>6.762</v>
       </c>
       <c r="Q4" t="n">
-        <v>-4.153799999999999</v>
+        <v>-8.860199999999999</v>
       </c>
       <c r="R4" t="n">
-        <v>3.4614</v>
+        <v>15.6222</v>
       </c>
       <c r="S4" t="n">
-        <v>1.3773</v>
+        <v>2.2132</v>
       </c>
       <c r="T4" t="n">
-        <v>-0.1803</v>
+        <v>-0.3649000000000001</v>
       </c>
       <c r="U4" t="n">
-        <v>1.5573</v>
+        <v>2.5781</v>
       </c>
       <c r="V4" t="n">
-        <v>3.231</v>
+        <v>12.3497</v>
       </c>
       <c r="W4" t="n">
-        <v>3.231</v>
+        <v>17.6266</v>
       </c>
       <c r="X4" t="n">
-        <v>0</v>
+        <v>-5.2763</v>
       </c>
     </row>
     <row r="5">
@@ -796,76 +796,76 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D5" t="n">
-        <v>18.5106</v>
+        <v>23.9763</v>
       </c>
       <c r="E5" t="n">
-        <v>6.530099999999999</v>
+        <v>11.2274</v>
       </c>
       <c r="F5" t="n">
-        <v>11.9808</v>
+        <v>12.7484</v>
       </c>
       <c r="G5" t="n">
-        <v>19.5501</v>
+        <v>22.5704</v>
       </c>
       <c r="H5" t="n">
-        <v>5.478</v>
+        <v>6.444600000000001</v>
       </c>
       <c r="I5" t="n">
-        <v>14.0727</v>
+        <v>16.1261</v>
       </c>
       <c r="J5" t="n">
-        <v>11.2305</v>
+        <v>14.2609</v>
       </c>
       <c r="K5" t="n">
-        <v>8.0808</v>
+        <v>7.976699999999999</v>
       </c>
       <c r="L5" t="n">
-        <v>3.1494</v>
+        <v>6.284199999999999</v>
       </c>
       <c r="M5" t="n">
-        <v>8.3202</v>
+        <v>8.309799999999999</v>
       </c>
       <c r="N5" t="n">
-        <v>-2.6037</v>
+        <v>-1.5321</v>
       </c>
       <c r="O5" t="n">
-        <v>10.923</v>
+        <v>9.841899999999999</v>
       </c>
       <c r="P5" t="n">
-        <v>5.538</v>
+        <v>8.1607</v>
       </c>
       <c r="Q5" t="n">
-        <v>-6.9228</v>
+        <v>-6.9948</v>
       </c>
       <c r="R5" t="n">
-        <v>12.4608</v>
+        <v>15.1555</v>
       </c>
       <c r="S5" t="n">
-        <v>1.5</v>
+        <v>1.3871</v>
       </c>
       <c r="T5" t="n">
-        <v>-1.0086</v>
+        <v>-0.3075000000000001</v>
       </c>
       <c r="U5" t="n">
-        <v>2.5083</v>
+        <v>1.6946</v>
       </c>
       <c r="V5" t="n">
-        <v>-8.077500000000001</v>
+        <v>-8.1425</v>
       </c>
       <c r="W5" t="n">
-        <v>3.231</v>
+        <v>4.2692</v>
       </c>
       <c r="X5" t="n">
-        <v>-11.3085</v>
+        <v>-12.4117</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Y. FALL</t>
+          <t>W. CLYBURN</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -874,76 +874,76 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D6" t="n">
-        <v>17.85</v>
+        <v>22.3621</v>
       </c>
       <c r="E6" t="n">
-        <v>8.5785</v>
+        <v>14.4605</v>
       </c>
       <c r="F6" t="n">
-        <v>9.2715</v>
+        <v>7.901599999999999</v>
       </c>
       <c r="G6" t="n">
-        <v>9.6828</v>
+        <v>20.1479</v>
       </c>
       <c r="H6" t="n">
-        <v>6.6006</v>
+        <v>-1.183400000000001</v>
       </c>
       <c r="I6" t="n">
-        <v>3.0822</v>
+        <v>21.3316</v>
       </c>
       <c r="J6" t="n">
-        <v>7.4811</v>
+        <v>24.1062</v>
       </c>
       <c r="K6" t="n">
-        <v>6.1515</v>
+        <v>-0.6800000000000005</v>
       </c>
       <c r="L6" t="n">
-        <v>1.3293</v>
+        <v>24.7858</v>
       </c>
       <c r="M6" t="n">
-        <v>2.2017</v>
+        <v>-3.958</v>
       </c>
       <c r="N6" t="n">
-        <v>0.4488000000000002</v>
+        <v>-0.5035000000000001</v>
       </c>
       <c r="O6" t="n">
-        <v>1.7526</v>
+        <v>-3.4545</v>
       </c>
       <c r="P6" t="n">
-        <v>4.8456</v>
+        <v>-2.0987</v>
       </c>
       <c r="Q6" t="n">
-        <v>-4.8462</v>
+        <v>-19.8191</v>
       </c>
       <c r="R6" t="n">
-        <v>9.691800000000001</v>
+        <v>17.7207</v>
       </c>
       <c r="S6" t="n">
-        <v>3.7602</v>
+        <v>5.7154</v>
       </c>
       <c r="T6" t="n">
-        <v>-0.5184</v>
+        <v>-0.2556999999999999</v>
       </c>
       <c r="U6" t="n">
-        <v>4.2786</v>
+        <v>5.9711</v>
       </c>
       <c r="V6" t="n">
-        <v>-0.4386</v>
+        <v>-1.402500000000001</v>
       </c>
       <c r="W6" t="n">
-        <v>6.462</v>
+        <v>10.4297</v>
       </c>
       <c r="X6" t="n">
-        <v>-6.9006</v>
+        <v>-11.8322</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>J. VESELY</t>
+          <t>Y. FALL</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -952,76 +952,76 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D7" t="n">
-        <v>17.1486</v>
+        <v>21.9728</v>
       </c>
       <c r="E7" t="n">
-        <v>9.5943</v>
+        <v>12.5153</v>
       </c>
       <c r="F7" t="n">
-        <v>7.5543</v>
+        <v>9.457100000000001</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.1289999999999991</v>
+        <v>12.2205</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.3170999999999998</v>
+        <v>9.5913</v>
       </c>
       <c r="I7" t="n">
-        <v>0.1877999999999997</v>
+        <v>2.6292</v>
       </c>
       <c r="J7" t="n">
-        <v>1.318500000000001</v>
+        <v>10.3235</v>
       </c>
       <c r="K7" t="n">
-        <v>-1.2531</v>
+        <v>8.6363</v>
       </c>
       <c r="L7" t="n">
-        <v>2.5716</v>
+        <v>1.6871</v>
       </c>
       <c r="M7" t="n">
-        <v>-1.4478</v>
+        <v>1.897</v>
       </c>
       <c r="N7" t="n">
-        <v>0.9363</v>
+        <v>0.9551999999999998</v>
       </c>
       <c r="O7" t="n">
-        <v>-2.383799999999999</v>
+        <v>0.9418</v>
       </c>
       <c r="P7" t="n">
-        <v>4.8459</v>
+        <v>5.8292</v>
       </c>
       <c r="Q7" t="n">
-        <v>-7.6152</v>
+        <v>-5.129799999999999</v>
       </c>
       <c r="R7" t="n">
-        <v>12.4608</v>
+        <v>10.9587</v>
       </c>
       <c r="S7" t="n">
-        <v>1.7016</v>
+        <v>6.6673</v>
       </c>
       <c r="T7" t="n">
-        <v>-0.7020000000000001</v>
+        <v>1.4354</v>
       </c>
       <c r="U7" t="n">
-        <v>2.4039</v>
+        <v>5.2315</v>
       </c>
       <c r="V7" t="n">
-        <v>10.7304</v>
+        <v>-2.7445</v>
       </c>
       <c r="W7" t="n">
-        <v>16.5936</v>
+        <v>5.885599999999999</v>
       </c>
       <c r="X7" t="n">
-        <v>-5.8626</v>
+        <v>-8.630199999999999</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>K. PUNTER</t>
+          <t>T. SHENGELIA</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1030,76 +1030,76 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D8" t="n">
-        <v>11.1192</v>
+        <v>18.1699</v>
       </c>
       <c r="E8" t="n">
-        <v>5.033399999999999</v>
+        <v>18.9358</v>
       </c>
       <c r="F8" t="n">
-        <v>6.0858</v>
+        <v>-0.766</v>
       </c>
       <c r="G8" t="n">
-        <v>4.9614</v>
+        <v>4.154499999999999</v>
       </c>
       <c r="H8" t="n">
-        <v>-3.582</v>
+        <v>10.4646</v>
       </c>
       <c r="I8" t="n">
-        <v>8.5434</v>
+        <v>-6.309899999999999</v>
       </c>
       <c r="J8" t="n">
-        <v>9.5397</v>
+        <v>15.6909</v>
       </c>
       <c r="K8" t="n">
-        <v>-2.986199999999999</v>
+        <v>10.9878</v>
       </c>
       <c r="L8" t="n">
-        <v>12.5259</v>
+        <v>4.7028</v>
       </c>
       <c r="M8" t="n">
-        <v>-4.5783</v>
+        <v>-11.5366</v>
       </c>
       <c r="N8" t="n">
-        <v>-0.5957999999999999</v>
+        <v>-0.5236000000000001</v>
       </c>
       <c r="O8" t="n">
-        <v>-3.9819</v>
+        <v>-11.0128</v>
       </c>
       <c r="P8" t="n">
-        <v>-0.0002999999999997449</v>
+        <v>-10.026</v>
       </c>
       <c r="Q8" t="n">
-        <v>-12.4608</v>
+        <v>-22.151</v>
       </c>
       <c r="R8" t="n">
-        <v>12.4608</v>
+        <v>12.1248</v>
       </c>
       <c r="S8" t="n">
-        <v>0.5732999999999999</v>
+        <v>7.4214</v>
       </c>
       <c r="T8" t="n">
-        <v>-0.5616</v>
+        <v>2.2802</v>
       </c>
       <c r="U8" t="n">
-        <v>1.1346</v>
+        <v>5.1415</v>
       </c>
       <c r="V8" t="n">
-        <v>5.5848</v>
+        <v>16.6203</v>
       </c>
       <c r="W8" t="n">
-        <v>8.5161</v>
+        <v>23.116</v>
       </c>
       <c r="X8" t="n">
-        <v>-2.9313</v>
+        <v>-6.495699999999999</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>T. SHENGELIA</t>
+          <t>M. CALE</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1108,70 +1108,70 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D9" t="n">
-        <v>11.1048</v>
+        <v>8.878300000000001</v>
       </c>
       <c r="E9" t="n">
-        <v>14.2014</v>
+        <v>1.4718</v>
       </c>
       <c r="F9" t="n">
-        <v>-3.0963</v>
+        <v>7.406099999999999</v>
       </c>
       <c r="G9" t="n">
-        <v>0.4014000000000002</v>
+        <v>14.3905</v>
       </c>
       <c r="H9" t="n">
-        <v>8.926500000000001</v>
+        <v>0.6024000000000002</v>
       </c>
       <c r="I9" t="n">
-        <v>-8.525400000000001</v>
+        <v>13.7881</v>
       </c>
       <c r="J9" t="n">
-        <v>11.8188</v>
+        <v>11.4765</v>
       </c>
       <c r="K9" t="n">
-        <v>8.4954</v>
+        <v>1.1625</v>
       </c>
       <c r="L9" t="n">
-        <v>3.3234</v>
+        <v>10.314</v>
       </c>
       <c r="M9" t="n">
-        <v>-11.4174</v>
+        <v>2.9139</v>
       </c>
       <c r="N9" t="n">
-        <v>0.4311000000000001</v>
+        <v>-0.5601000000000002</v>
       </c>
       <c r="O9" t="n">
-        <v>-11.8485</v>
+        <v>3.474</v>
       </c>
       <c r="P9" t="n">
-        <v>-9.691800000000001</v>
+        <v>-3.7308</v>
       </c>
       <c r="Q9" t="n">
-        <v>-19.3836</v>
+        <v>-10.4922</v>
       </c>
       <c r="R9" t="n">
-        <v>9.691800000000001</v>
+        <v>6.762</v>
       </c>
       <c r="S9" t="n">
-        <v>4.9791</v>
+        <v>-0.4706</v>
       </c>
       <c r="T9" t="n">
-        <v>1.0644</v>
+        <v>-1.4031</v>
       </c>
       <c r="U9" t="n">
-        <v>3.9144</v>
+        <v>0.9324000000000001</v>
       </c>
       <c r="V9" t="n">
-        <v>15.4167</v>
+        <v>-1.3111</v>
       </c>
       <c r="W9" t="n">
-        <v>20.7018</v>
+        <v>1.8908</v>
       </c>
       <c r="X9" t="n">
-        <v>-5.2851</v>
+        <v>-3.2019</v>
       </c>
     </row>
     <row r="10">
@@ -1186,76 +1186,76 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D10" t="n">
-        <v>5.9319</v>
+        <v>8.7293</v>
       </c>
       <c r="E10" t="n">
-        <v>-4.719</v>
+        <v>-4.8259</v>
       </c>
       <c r="F10" t="n">
-        <v>10.6512</v>
+        <v>13.5555</v>
       </c>
       <c r="G10" t="n">
-        <v>6.2016</v>
+        <v>11.1963</v>
       </c>
       <c r="H10" t="n">
-        <v>-9.581399999999999</v>
+        <v>-6.1441</v>
       </c>
       <c r="I10" t="n">
-        <v>15.783</v>
+        <v>17.3404</v>
       </c>
       <c r="J10" t="n">
-        <v>6.351</v>
+        <v>9.440899999999999</v>
       </c>
       <c r="K10" t="n">
-        <v>-5.968500000000001</v>
+        <v>-2.4168</v>
       </c>
       <c r="L10" t="n">
-        <v>12.3195</v>
+        <v>11.8584</v>
       </c>
       <c r="M10" t="n">
-        <v>-0.1496999999999998</v>
+        <v>1.755099999999999</v>
       </c>
       <c r="N10" t="n">
-        <v>-3.6129</v>
+        <v>-3.7269</v>
       </c>
       <c r="O10" t="n">
-        <v>3.4635</v>
+        <v>5.482</v>
       </c>
       <c r="P10" t="n">
-        <v>-0.6924000000000001</v>
+        <v>-1.6323</v>
       </c>
       <c r="Q10" t="n">
-        <v>-11.7684</v>
+        <v>-15.3892</v>
       </c>
       <c r="R10" t="n">
-        <v>11.0763</v>
+        <v>13.7566</v>
       </c>
       <c r="S10" t="n">
-        <v>-0.4544999999999999</v>
+        <v>-0.5914000000000001</v>
       </c>
       <c r="T10" t="n">
-        <v>-3.4098</v>
+        <v>-2.9039</v>
       </c>
       <c r="U10" t="n">
-        <v>2.9556</v>
+        <v>2.3123</v>
       </c>
       <c r="V10" t="n">
-        <v>0.8772000000000002</v>
+        <v>-0.2435000000000005</v>
       </c>
       <c r="W10" t="n">
-        <v>4.1082</v>
+        <v>4.0257</v>
       </c>
       <c r="X10" t="n">
-        <v>-3.231</v>
+        <v>-4.2692</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>M. CALE</t>
+          <t>K. PUNTER</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1264,70 +1264,70 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D11" t="n">
-        <v>4.580700000000001</v>
+        <v>4.780100000000001</v>
       </c>
       <c r="E11" t="n">
-        <v>0.6050999999999997</v>
+        <v>0.6221999999999996</v>
       </c>
       <c r="F11" t="n">
-        <v>3.975299999999999</v>
+        <v>4.1581</v>
       </c>
       <c r="G11" t="n">
-        <v>13.4535</v>
+        <v>0.1347999999999989</v>
       </c>
       <c r="H11" t="n">
-        <v>-2.3172</v>
+        <v>-6.4969</v>
       </c>
       <c r="I11" t="n">
-        <v>15.7707</v>
+        <v>6.6323</v>
       </c>
       <c r="J11" t="n">
-        <v>12.2784</v>
+        <v>6.8047</v>
       </c>
       <c r="K11" t="n">
-        <v>-0.2391</v>
+        <v>-4.8271</v>
       </c>
       <c r="L11" t="n">
-        <v>12.5175</v>
+        <v>11.6321</v>
       </c>
       <c r="M11" t="n">
-        <v>1.1751</v>
+        <v>-6.6699</v>
       </c>
       <c r="N11" t="n">
-        <v>-2.0781</v>
+        <v>-1.6699</v>
       </c>
       <c r="O11" t="n">
-        <v>3.253200000000001</v>
+        <v>-4.9998</v>
       </c>
       <c r="P11" t="n">
-        <v>-5.5383</v>
+        <v>-0.6994999999999998</v>
       </c>
       <c r="Q11" t="n">
-        <v>-10.3842</v>
+        <v>-15.1558</v>
       </c>
       <c r="R11" t="n">
-        <v>4.8459</v>
+        <v>14.4564</v>
       </c>
       <c r="S11" t="n">
-        <v>-0.9810000000000001</v>
+        <v>0.9077000000000001</v>
       </c>
       <c r="T11" t="n">
-        <v>-2.1663</v>
+        <v>-0.6481</v>
       </c>
       <c r="U11" t="n">
-        <v>1.1853</v>
+        <v>1.5557</v>
       </c>
       <c r="V11" t="n">
-        <v>-2.3538</v>
+        <v>4.4368</v>
       </c>
       <c r="W11" t="n">
-        <v>0.8772</v>
+        <v>9.6211</v>
       </c>
       <c r="X11" t="n">
-        <v>-3.231</v>
+        <v>-5.1846</v>
       </c>
     </row>
     <row r="12">
@@ -1342,70 +1342,70 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D12" t="n">
-        <v>0.2325</v>
+        <v>0.7706000000000004</v>
       </c>
       <c r="E12" t="n">
-        <v>-6.1275</v>
+        <v>-4.9995</v>
       </c>
       <c r="F12" t="n">
-        <v>6.36</v>
+        <v>5.7704</v>
       </c>
       <c r="G12" t="n">
-        <v>9.274800000000001</v>
+        <v>9.9842</v>
       </c>
       <c r="H12" t="n">
-        <v>5.9499</v>
+        <v>6.1067</v>
       </c>
       <c r="I12" t="n">
-        <v>3.3246</v>
+        <v>3.877200000000001</v>
       </c>
       <c r="J12" t="n">
-        <v>9.184200000000001</v>
+        <v>11.8903</v>
       </c>
       <c r="K12" t="n">
-        <v>2.4666</v>
+        <v>3.1409</v>
       </c>
       <c r="L12" t="n">
-        <v>6.7176</v>
+        <v>8.749599999999999</v>
       </c>
       <c r="M12" t="n">
-        <v>0.09030000000000005</v>
+        <v>-1.9067</v>
       </c>
       <c r="N12" t="n">
-        <v>3.4836</v>
+        <v>2.9661</v>
       </c>
       <c r="O12" t="n">
-        <v>-3.393</v>
+        <v>-4.8728</v>
       </c>
       <c r="P12" t="n">
-        <v>-4.8456</v>
+        <v>-4.8966</v>
       </c>
       <c r="Q12" t="n">
-        <v>-13.8453</v>
+        <v>-15.156</v>
       </c>
       <c r="R12" t="n">
-        <v>8.999700000000001</v>
+        <v>10.2594</v>
       </c>
       <c r="S12" t="n">
-        <v>1.0887</v>
+        <v>1.2493</v>
       </c>
       <c r="T12" t="n">
-        <v>-1.4667</v>
+        <v>-1.7341</v>
       </c>
       <c r="U12" t="n">
-        <v>2.5554</v>
+        <v>2.983</v>
       </c>
       <c r="V12" t="n">
-        <v>-5.2851</v>
+        <v>-5.5657</v>
       </c>
       <c r="W12" t="n">
         <v>0</v>
       </c>
       <c r="X12" t="n">
-        <v>-5.2851</v>
+        <v>-5.5657</v>
       </c>
     </row>
     <row r="13">
@@ -1420,70 +1420,70 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D13" t="n">
-        <v>-1.3899</v>
+        <v>-1.5241</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.4742999999999999</v>
+        <v>-0.6511</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.9153</v>
+        <v>-0.8729999999999999</v>
       </c>
       <c r="G13" t="n">
-        <v>-2.463</v>
+        <v>-2.4572</v>
       </c>
       <c r="H13" t="n">
-        <v>-2.8821</v>
+        <v>-3.6083</v>
       </c>
       <c r="I13" t="n">
-        <v>0.4194</v>
+        <v>1.1511</v>
       </c>
       <c r="J13" t="n">
-        <v>-0.7377</v>
+        <v>-1.6052</v>
       </c>
       <c r="K13" t="n">
-        <v>-0.8484</v>
+        <v>-1.7887</v>
       </c>
       <c r="L13" t="n">
-        <v>0.1107</v>
+        <v>0.1835</v>
       </c>
       <c r="M13" t="n">
-        <v>-1.7253</v>
+        <v>-0.8519</v>
       </c>
       <c r="N13" t="n">
-        <v>-2.0337</v>
+        <v>-1.8199</v>
       </c>
       <c r="O13" t="n">
-        <v>0.3084</v>
+        <v>0.9676</v>
       </c>
       <c r="P13" t="n">
-        <v>0</v>
+        <v>0.6995</v>
       </c>
       <c r="Q13" t="n">
         <v>0</v>
       </c>
       <c r="R13" t="n">
-        <v>0</v>
+        <v>0.6995</v>
       </c>
       <c r="S13" t="n">
-        <v>1.9506</v>
+        <v>2.1247</v>
       </c>
       <c r="T13" t="n">
-        <v>0.2634</v>
+        <v>0.9542</v>
       </c>
       <c r="U13" t="n">
-        <v>1.6872</v>
+        <v>1.1708</v>
       </c>
       <c r="V13" t="n">
-        <v>-0.8772</v>
+        <v>-1.8911</v>
       </c>
       <c r="W13" t="n">
         <v>0</v>
       </c>
       <c r="X13" t="n">
-        <v>-0.8772</v>
+        <v>-1.8911</v>
       </c>
     </row>
     <row r="14">
@@ -1498,70 +1498,70 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D14" t="n">
-        <v>149.6145</v>
+        <v>191.645</v>
       </c>
       <c r="E14" t="n">
-        <v>67.5903</v>
+        <v>95.17490000000001</v>
       </c>
       <c r="F14" t="n">
-        <v>82.02510000000001</v>
+        <v>96.46899999999999</v>
       </c>
       <c r="G14" t="n">
-        <v>121.401</v>
+        <v>151.1125</v>
       </c>
       <c r="H14" t="n">
-        <v>28.0146</v>
+        <v>43.3006</v>
       </c>
       <c r="I14" t="n">
-        <v>93.38639999999999</v>
+        <v>107.8134</v>
       </c>
       <c r="J14" t="n">
-        <v>126.2724</v>
+        <v>156.7391</v>
       </c>
       <c r="K14" t="n">
-        <v>33.7974</v>
+        <v>48.57319999999999</v>
       </c>
       <c r="L14" t="n">
-        <v>92.4744</v>
+        <v>108.1664</v>
       </c>
       <c r="M14" t="n">
-        <v>-4.871400000000001</v>
+        <v>-5.627300000000001</v>
       </c>
       <c r="N14" t="n">
-        <v>-5.783099999999999</v>
+        <v>-5.273099999999999</v>
       </c>
       <c r="O14" t="n">
-        <v>0.9120000000000019</v>
+        <v>-0.3539000000000021</v>
       </c>
       <c r="P14" t="n">
-        <v>-13.8468</v>
+        <v>-10.4926</v>
       </c>
       <c r="Q14" t="n">
-        <v>-124.6089</v>
+        <v>-146.895</v>
       </c>
       <c r="R14" t="n">
-        <v>110.763</v>
+        <v>136.4023</v>
       </c>
       <c r="S14" t="n">
-        <v>21.1989</v>
+        <v>30.9137</v>
       </c>
       <c r="T14" t="n">
-        <v>-12.0339</v>
+        <v>-3.686</v>
       </c>
       <c r="U14" t="n">
-        <v>33.2316</v>
+        <v>34.5992</v>
       </c>
       <c r="V14" t="n">
-        <v>20.8623</v>
+        <v>20.1108</v>
       </c>
       <c r="W14" t="n">
-        <v>77.9607</v>
+        <v>89.01690000000001</v>
       </c>
       <c r="X14" t="n">
-        <v>-57.0981</v>
+        <v>-68.90609999999998</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
new acb playoffs games
</commit_message>
<xml_diff>
--- a/informes_data/ACB/2025-26/playoffs/aggregate_individual/AGG_IND_Barça.xlsx
+++ b/informes_data/ACB/2025-26/playoffs/aggregate_individual/AGG_IND_Barça.xlsx
@@ -562,76 +562,76 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="D2" t="n">
-        <v>33.7133</v>
+        <v>23.7981</v>
       </c>
       <c r="E2" t="n">
-        <v>12.9768</v>
+        <v>14.3693</v>
       </c>
       <c r="F2" t="n">
-        <v>20.7364</v>
+        <v>9.428800000000001</v>
       </c>
       <c r="G2" t="n">
-        <v>30.2633</v>
+        <v>23.1843</v>
       </c>
       <c r="H2" t="n">
-        <v>19.8114</v>
+        <v>9.1592</v>
       </c>
       <c r="I2" t="n">
-        <v>10.4519</v>
+        <v>14.0251</v>
       </c>
       <c r="J2" t="n">
-        <v>25.0465</v>
+        <v>19.4604</v>
       </c>
       <c r="K2" t="n">
-        <v>20.3654</v>
+        <v>8.2652</v>
       </c>
       <c r="L2" t="n">
-        <v>4.6811</v>
+        <v>11.195</v>
       </c>
       <c r="M2" t="n">
-        <v>5.2166</v>
+        <v>3.7238</v>
       </c>
       <c r="N2" t="n">
-        <v>-0.5542999999999999</v>
+        <v>0.8938999999999999</v>
       </c>
       <c r="O2" t="n">
-        <v>5.7709</v>
+        <v>2.8299</v>
       </c>
       <c r="P2" t="n">
-        <v>-3.4975</v>
+        <v>-0.2295</v>
       </c>
       <c r="Q2" t="n">
-        <v>-17.4876</v>
+        <v>-5.7375</v>
       </c>
       <c r="R2" t="n">
-        <v>13.9901</v>
+        <v>5.508</v>
       </c>
       <c r="S2" t="n">
-        <v>2.1447</v>
+        <v>0.3025</v>
       </c>
       <c r="T2" t="n">
-        <v>-1.3979</v>
+        <v>-0.9765999999999999</v>
       </c>
       <c r="U2" t="n">
-        <v>3.5426</v>
+        <v>1.2792</v>
       </c>
       <c r="V2" t="n">
-        <v>4.803</v>
+        <v>0.541</v>
       </c>
       <c r="W2" t="n">
-        <v>6.8156</v>
+        <v>1.623</v>
       </c>
       <c r="X2" t="n">
-        <v>-2.0129</v>
+        <v>-1.082</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>N. LAPROVITTOLA</t>
+          <t>J. VESELY</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -640,76 +640,76 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D3" t="n">
-        <v>25.3924</v>
+        <v>10.4631</v>
       </c>
       <c r="E3" t="n">
-        <v>19.7664</v>
+        <v>3.0499</v>
       </c>
       <c r="F3" t="n">
-        <v>5.625599999999999</v>
+        <v>7.413200000000001</v>
       </c>
       <c r="G3" t="n">
-        <v>25.4082</v>
+        <v>1.6255</v>
       </c>
       <c r="H3" t="n">
-        <v>4.1893</v>
+        <v>1.6015</v>
       </c>
       <c r="I3" t="n">
-        <v>21.2189</v>
+        <v>0.02400000000000002</v>
       </c>
       <c r="J3" t="n">
-        <v>24.0299</v>
+        <v>1.462</v>
       </c>
       <c r="K3" t="n">
-        <v>2.8042</v>
+        <v>1.2633</v>
       </c>
       <c r="L3" t="n">
-        <v>21.2257</v>
+        <v>0.1987</v>
       </c>
       <c r="M3" t="n">
-        <v>1.3783</v>
+        <v>0.1634999999999999</v>
       </c>
       <c r="N3" t="n">
-        <v>1.3852</v>
+        <v>0.3382000000000001</v>
       </c>
       <c r="O3" t="n">
-        <v>-0.006800000000000028</v>
+        <v>-0.1747000000000001</v>
       </c>
       <c r="P3" t="n">
-        <v>-5.3626</v>
+        <v>0.459</v>
       </c>
       <c r="Q3" t="n">
-        <v>-10.2593</v>
+        <v>-4.59</v>
       </c>
       <c r="R3" t="n">
-        <v>4.8964</v>
+        <v>5.048999999999999</v>
       </c>
       <c r="S3" t="n">
-        <v>2.1449</v>
+        <v>0.7786</v>
       </c>
       <c r="T3" t="n">
-        <v>0.6594</v>
+        <v>-0.3142</v>
       </c>
       <c r="U3" t="n">
-        <v>1.4856</v>
+        <v>1.0928</v>
       </c>
       <c r="V3" t="n">
-        <v>3.2019</v>
+        <v>7.600000000000001</v>
       </c>
       <c r="W3" t="n">
-        <v>5.3366</v>
+        <v>6.492000000000001</v>
       </c>
       <c r="X3" t="n">
-        <v>-2.1346</v>
+        <v>1.108</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>J. VESELY</t>
+          <t>J. PARRA</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -718,76 +718,76 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="D4" t="n">
-        <v>24.424</v>
+        <v>10.3781</v>
       </c>
       <c r="E4" t="n">
-        <v>13.6752</v>
+        <v>5.423</v>
       </c>
       <c r="F4" t="n">
-        <v>10.7488</v>
+        <v>4.955</v>
       </c>
       <c r="G4" t="n">
-        <v>3.0991</v>
+        <v>11.7441</v>
       </c>
       <c r="H4" t="n">
-        <v>3.523000000000001</v>
+        <v>2.811</v>
       </c>
       <c r="I4" t="n">
-        <v>-0.4235000000000002</v>
+        <v>8.933199999999999</v>
       </c>
       <c r="J4" t="n">
-        <v>5.273999999999999</v>
+        <v>6.1299</v>
       </c>
       <c r="K4" t="n">
-        <v>3.212</v>
+        <v>2.3376</v>
       </c>
       <c r="L4" t="n">
-        <v>2.0621</v>
+        <v>3.7925</v>
       </c>
       <c r="M4" t="n">
-        <v>-2.1749</v>
+        <v>5.6142</v>
       </c>
       <c r="N4" t="n">
-        <v>0.3107000000000002</v>
+        <v>0.4734000000000002</v>
       </c>
       <c r="O4" t="n">
-        <v>-2.4854</v>
+        <v>5.1408</v>
       </c>
       <c r="P4" t="n">
-        <v>6.762</v>
+        <v>5.049</v>
       </c>
       <c r="Q4" t="n">
-        <v>-8.860199999999999</v>
+        <v>-1.1475</v>
       </c>
       <c r="R4" t="n">
-        <v>15.6222</v>
+        <v>6.1965</v>
       </c>
       <c r="S4" t="n">
-        <v>2.2132</v>
+        <v>-0.8541000000000001</v>
       </c>
       <c r="T4" t="n">
-        <v>-0.3649000000000001</v>
+        <v>-0.6415000000000001</v>
       </c>
       <c r="U4" t="n">
-        <v>2.5781</v>
+        <v>-0.2126000000000001</v>
       </c>
       <c r="V4" t="n">
-        <v>12.3497</v>
+        <v>-5.5609</v>
       </c>
       <c r="W4" t="n">
-        <v>17.6266</v>
+        <v>1.082</v>
       </c>
       <c r="X4" t="n">
-        <v>-5.2763</v>
+        <v>-6.6429</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>J. PARRA</t>
+          <t>Y. FALL</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -796,76 +796,76 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="D5" t="n">
-        <v>23.9763</v>
+        <v>9.0128</v>
       </c>
       <c r="E5" t="n">
-        <v>11.2274</v>
+        <v>4.6071</v>
       </c>
       <c r="F5" t="n">
-        <v>12.7484</v>
+        <v>4.405600000000001</v>
       </c>
       <c r="G5" t="n">
-        <v>22.5704</v>
+        <v>5.5922</v>
       </c>
       <c r="H5" t="n">
-        <v>6.444600000000001</v>
+        <v>4.0927</v>
       </c>
       <c r="I5" t="n">
-        <v>16.1261</v>
+        <v>1.4995</v>
       </c>
       <c r="J5" t="n">
-        <v>14.2609</v>
+        <v>3.212</v>
       </c>
       <c r="K5" t="n">
-        <v>7.976699999999999</v>
+        <v>2.508</v>
       </c>
       <c r="L5" t="n">
-        <v>6.284199999999999</v>
+        <v>0.704</v>
       </c>
       <c r="M5" t="n">
-        <v>8.309799999999999</v>
+        <v>2.38</v>
       </c>
       <c r="N5" t="n">
-        <v>-1.5321</v>
+        <v>1.5847</v>
       </c>
       <c r="O5" t="n">
-        <v>9.841899999999999</v>
+        <v>0.7954999999999999</v>
       </c>
       <c r="P5" t="n">
-        <v>8.1607</v>
+        <v>2.5245</v>
       </c>
       <c r="Q5" t="n">
-        <v>-6.9948</v>
+        <v>-1.6065</v>
       </c>
       <c r="R5" t="n">
-        <v>15.1555</v>
+        <v>4.131</v>
       </c>
       <c r="S5" t="n">
-        <v>1.3871</v>
+        <v>2.5192</v>
       </c>
       <c r="T5" t="n">
-        <v>-0.3075000000000001</v>
+        <v>0.536</v>
       </c>
       <c r="U5" t="n">
-        <v>1.6946</v>
+        <v>1.9832</v>
       </c>
       <c r="V5" t="n">
-        <v>-8.1425</v>
+        <v>-1.6231</v>
       </c>
       <c r="W5" t="n">
-        <v>4.2692</v>
+        <v>2.4657</v>
       </c>
       <c r="X5" t="n">
-        <v>-12.4117</v>
+        <v>-4.0888</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>W. CLYBURN</t>
+          <t>M. CALE</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -874,76 +874,76 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="D6" t="n">
-        <v>22.3621</v>
+        <v>8.912800000000001</v>
       </c>
       <c r="E6" t="n">
-        <v>14.4605</v>
+        <v>3.0085</v>
       </c>
       <c r="F6" t="n">
-        <v>7.901599999999999</v>
+        <v>5.9043</v>
       </c>
       <c r="G6" t="n">
-        <v>20.1479</v>
+        <v>8.039999999999999</v>
       </c>
       <c r="H6" t="n">
-        <v>-1.183400000000001</v>
+        <v>1.63</v>
       </c>
       <c r="I6" t="n">
-        <v>21.3316</v>
+        <v>6.410299999999999</v>
       </c>
       <c r="J6" t="n">
-        <v>24.1062</v>
+        <v>5.595199999999999</v>
       </c>
       <c r="K6" t="n">
-        <v>-0.6800000000000005</v>
+        <v>0.9507</v>
       </c>
       <c r="L6" t="n">
-        <v>24.7858</v>
+        <v>4.644600000000001</v>
       </c>
       <c r="M6" t="n">
-        <v>-3.958</v>
+        <v>2.4449</v>
       </c>
       <c r="N6" t="n">
-        <v>-0.5035000000000001</v>
+        <v>0.6792</v>
       </c>
       <c r="O6" t="n">
-        <v>-3.4545</v>
+        <v>1.7655</v>
       </c>
       <c r="P6" t="n">
-        <v>-2.0987</v>
+        <v>-0.2295</v>
       </c>
       <c r="Q6" t="n">
-        <v>-19.8191</v>
+        <v>-3.4425</v>
       </c>
       <c r="R6" t="n">
-        <v>17.7207</v>
+        <v>3.213</v>
       </c>
       <c r="S6" t="n">
-        <v>5.7154</v>
+        <v>-0.2817</v>
       </c>
       <c r="T6" t="n">
-        <v>-0.2556999999999999</v>
+        <v>-0.5281</v>
       </c>
       <c r="U6" t="n">
-        <v>5.9711</v>
+        <v>0.2465000000000001</v>
       </c>
       <c r="V6" t="n">
-        <v>-1.402500000000001</v>
+        <v>1.3837</v>
       </c>
       <c r="W6" t="n">
-        <v>10.4297</v>
+        <v>1.3837</v>
       </c>
       <c r="X6" t="n">
-        <v>-11.8322</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Y. FALL</t>
+          <t>T. SATORANSKY</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -952,70 +952,70 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="D7" t="n">
-        <v>21.9728</v>
+        <v>6.892</v>
       </c>
       <c r="E7" t="n">
-        <v>12.5153</v>
+        <v>1.6555</v>
       </c>
       <c r="F7" t="n">
-        <v>9.457100000000001</v>
+        <v>5.236499999999999</v>
       </c>
       <c r="G7" t="n">
-        <v>12.2205</v>
+        <v>9.4642</v>
       </c>
       <c r="H7" t="n">
-        <v>9.5913</v>
+        <v>1.7775</v>
       </c>
       <c r="I7" t="n">
-        <v>2.6292</v>
+        <v>7.6867</v>
       </c>
       <c r="J7" t="n">
-        <v>10.3235</v>
+        <v>8.168900000000001</v>
       </c>
       <c r="K7" t="n">
-        <v>8.6363</v>
+        <v>2.0859</v>
       </c>
       <c r="L7" t="n">
-        <v>1.6871</v>
+        <v>6.083</v>
       </c>
       <c r="M7" t="n">
-        <v>1.897</v>
+        <v>1.2954</v>
       </c>
       <c r="N7" t="n">
-        <v>0.9551999999999998</v>
+        <v>-0.3083999999999999</v>
       </c>
       <c r="O7" t="n">
-        <v>0.9418</v>
+        <v>1.604</v>
       </c>
       <c r="P7" t="n">
-        <v>5.8292</v>
+        <v>-1.377</v>
       </c>
       <c r="Q7" t="n">
-        <v>-5.129799999999999</v>
+        <v>-6.196400000000001</v>
       </c>
       <c r="R7" t="n">
-        <v>10.9587</v>
+        <v>4.8195</v>
       </c>
       <c r="S7" t="n">
-        <v>6.6673</v>
+        <v>-0.5659000000000001</v>
       </c>
       <c r="T7" t="n">
-        <v>1.4354</v>
+        <v>-1.8516</v>
       </c>
       <c r="U7" t="n">
-        <v>5.2315</v>
+        <v>1.2857</v>
       </c>
       <c r="V7" t="n">
-        <v>-2.7445</v>
+        <v>-0.6294999999999999</v>
       </c>
       <c r="W7" t="n">
-        <v>5.885599999999999</v>
+        <v>1.5347</v>
       </c>
       <c r="X7" t="n">
-        <v>-8.630199999999999</v>
+        <v>-2.164</v>
       </c>
     </row>
     <row r="8">
@@ -1030,76 +1030,76 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="D8" t="n">
-        <v>18.1699</v>
+        <v>6.4404</v>
       </c>
       <c r="E8" t="n">
-        <v>18.9358</v>
+        <v>4.439900000000001</v>
       </c>
       <c r="F8" t="n">
-        <v>-0.766</v>
+        <v>2.0005</v>
       </c>
       <c r="G8" t="n">
-        <v>4.154499999999999</v>
+        <v>3.184</v>
       </c>
       <c r="H8" t="n">
-        <v>10.4646</v>
+        <v>3.4464</v>
       </c>
       <c r="I8" t="n">
-        <v>-6.309899999999999</v>
+        <v>-0.2624000000000004</v>
       </c>
       <c r="J8" t="n">
-        <v>15.6909</v>
+        <v>6.5577</v>
       </c>
       <c r="K8" t="n">
-        <v>10.9878</v>
+        <v>2.9203</v>
       </c>
       <c r="L8" t="n">
-        <v>4.7028</v>
+        <v>3.6378</v>
       </c>
       <c r="M8" t="n">
-        <v>-11.5366</v>
+        <v>-3.373699999999999</v>
       </c>
       <c r="N8" t="n">
-        <v>-0.5236000000000001</v>
+        <v>0.5265</v>
       </c>
       <c r="O8" t="n">
-        <v>-11.0128</v>
+        <v>-3.9</v>
       </c>
       <c r="P8" t="n">
-        <v>-10.026</v>
+        <v>-4.8195</v>
       </c>
       <c r="Q8" t="n">
-        <v>-22.151</v>
+        <v>-8.491299999999999</v>
       </c>
       <c r="R8" t="n">
-        <v>12.1248</v>
+        <v>3.672</v>
       </c>
       <c r="S8" t="n">
-        <v>7.4214</v>
+        <v>3.2951</v>
       </c>
       <c r="T8" t="n">
-        <v>2.2802</v>
+        <v>0.36</v>
       </c>
       <c r="U8" t="n">
-        <v>5.1415</v>
+        <v>2.9351</v>
       </c>
       <c r="V8" t="n">
-        <v>16.6203</v>
+        <v>4.7807</v>
       </c>
       <c r="W8" t="n">
-        <v>23.116</v>
+        <v>6.0136</v>
       </c>
       <c r="X8" t="n">
-        <v>-6.495699999999999</v>
+        <v>-1.2329</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>M. CALE</t>
+          <t>W. CLYBURN</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1108,76 +1108,76 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="D9" t="n">
-        <v>8.878300000000001</v>
+        <v>4.4085</v>
       </c>
       <c r="E9" t="n">
-        <v>1.4718</v>
+        <v>-3.3131</v>
       </c>
       <c r="F9" t="n">
-        <v>7.406099999999999</v>
+        <v>7.7217</v>
       </c>
       <c r="G9" t="n">
-        <v>14.3905</v>
+        <v>-1.5211</v>
       </c>
       <c r="H9" t="n">
-        <v>0.6024000000000002</v>
+        <v>-3.3502</v>
       </c>
       <c r="I9" t="n">
-        <v>13.7881</v>
+        <v>1.8291</v>
       </c>
       <c r="J9" t="n">
-        <v>11.4765</v>
+        <v>-2.4166</v>
       </c>
       <c r="K9" t="n">
-        <v>1.1625</v>
+        <v>-4.1913</v>
       </c>
       <c r="L9" t="n">
-        <v>10.314</v>
+        <v>1.7747</v>
       </c>
       <c r="M9" t="n">
-        <v>2.9139</v>
+        <v>0.8955000000000001</v>
       </c>
       <c r="N9" t="n">
-        <v>-0.5601000000000002</v>
+        <v>0.8411000000000001</v>
       </c>
       <c r="O9" t="n">
-        <v>3.474</v>
+        <v>0.05439999999999989</v>
       </c>
       <c r="P9" t="n">
-        <v>-3.7308</v>
+        <v>0</v>
       </c>
       <c r="Q9" t="n">
-        <v>-10.4922</v>
+        <v>-6.1965</v>
       </c>
       <c r="R9" t="n">
-        <v>6.762</v>
+        <v>6.1965</v>
       </c>
       <c r="S9" t="n">
-        <v>-0.4706</v>
+        <v>2.6836</v>
       </c>
       <c r="T9" t="n">
-        <v>-1.4031</v>
+        <v>-0.4121</v>
       </c>
       <c r="U9" t="n">
-        <v>0.9324000000000001</v>
+        <v>3.0955</v>
       </c>
       <c r="V9" t="n">
-        <v>-1.3111</v>
+        <v>3.246</v>
       </c>
       <c r="W9" t="n">
-        <v>1.8908</v>
+        <v>5.7118</v>
       </c>
       <c r="X9" t="n">
-        <v>-3.2019</v>
+        <v>-2.4658</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>T. SATORANSKY</t>
+          <t>N. LAPROVITTOLA</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1186,76 +1186,76 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="D10" t="n">
-        <v>8.7293</v>
+        <v>3.574800000000001</v>
       </c>
       <c r="E10" t="n">
-        <v>-4.8259</v>
+        <v>3.3933</v>
       </c>
       <c r="F10" t="n">
-        <v>13.5555</v>
+        <v>0.1815</v>
       </c>
       <c r="G10" t="n">
-        <v>11.1963</v>
+        <v>5.9868</v>
       </c>
       <c r="H10" t="n">
-        <v>-6.1441</v>
+        <v>1.14</v>
       </c>
       <c r="I10" t="n">
-        <v>17.3404</v>
+        <v>4.8468</v>
       </c>
       <c r="J10" t="n">
-        <v>9.440899999999999</v>
+        <v>5.2463</v>
       </c>
       <c r="K10" t="n">
-        <v>-2.4168</v>
+        <v>0.7432000000000001</v>
       </c>
       <c r="L10" t="n">
-        <v>11.8584</v>
+        <v>4.5031</v>
       </c>
       <c r="M10" t="n">
-        <v>1.755099999999999</v>
+        <v>0.7407</v>
       </c>
       <c r="N10" t="n">
-        <v>-3.7269</v>
+        <v>0.3969</v>
       </c>
       <c r="O10" t="n">
-        <v>5.482</v>
+        <v>0.3437</v>
       </c>
       <c r="P10" t="n">
-        <v>-1.6323</v>
+        <v>-1.6065</v>
       </c>
       <c r="Q10" t="n">
-        <v>-15.3892</v>
+        <v>-2.295</v>
       </c>
       <c r="R10" t="n">
-        <v>13.7566</v>
+        <v>0.6885</v>
       </c>
       <c r="S10" t="n">
-        <v>-0.5914000000000001</v>
+        <v>0.2765</v>
       </c>
       <c r="T10" t="n">
-        <v>-2.9039</v>
+        <v>0.4420000000000001</v>
       </c>
       <c r="U10" t="n">
-        <v>2.3123</v>
+        <v>-0.1656</v>
       </c>
       <c r="V10" t="n">
-        <v>-0.2435000000000005</v>
+        <v>-1.082</v>
       </c>
       <c r="W10" t="n">
-        <v>4.0257</v>
+        <v>0</v>
       </c>
       <c r="X10" t="n">
-        <v>-4.2692</v>
+        <v>-1.082</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>K. PUNTER</t>
+          <t>J. MARCOS</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1264,76 +1264,76 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="D11" t="n">
-        <v>4.780100000000001</v>
+        <v>2.0093</v>
       </c>
       <c r="E11" t="n">
-        <v>0.6221999999999996</v>
+        <v>-2.6397</v>
       </c>
       <c r="F11" t="n">
-        <v>4.1581</v>
+        <v>4.649</v>
       </c>
       <c r="G11" t="n">
-        <v>0.1347999999999989</v>
+        <v>10.1335</v>
       </c>
       <c r="H11" t="n">
-        <v>-6.4969</v>
+        <v>4.0604</v>
       </c>
       <c r="I11" t="n">
-        <v>6.6323</v>
+        <v>6.072900000000001</v>
       </c>
       <c r="J11" t="n">
-        <v>6.8047</v>
+        <v>8.2561</v>
       </c>
       <c r="K11" t="n">
-        <v>-4.8271</v>
+        <v>2.3318</v>
       </c>
       <c r="L11" t="n">
-        <v>11.6321</v>
+        <v>5.924300000000001</v>
       </c>
       <c r="M11" t="n">
-        <v>-6.6699</v>
+        <v>1.8774</v>
       </c>
       <c r="N11" t="n">
-        <v>-1.6699</v>
+        <v>1.7286</v>
       </c>
       <c r="O11" t="n">
-        <v>-4.9998</v>
+        <v>0.1488</v>
       </c>
       <c r="P11" t="n">
-        <v>-0.6994999999999998</v>
+        <v>-5.7373</v>
       </c>
       <c r="Q11" t="n">
-        <v>-15.1558</v>
+        <v>-10.3273</v>
       </c>
       <c r="R11" t="n">
-        <v>14.4564</v>
+        <v>4.59</v>
       </c>
       <c r="S11" t="n">
-        <v>0.9077000000000001</v>
+        <v>1.3118</v>
       </c>
       <c r="T11" t="n">
-        <v>-0.6481</v>
+        <v>-0.5686</v>
       </c>
       <c r="U11" t="n">
-        <v>1.5557</v>
+        <v>1.8804</v>
       </c>
       <c r="V11" t="n">
-        <v>4.4368</v>
+        <v>-3.6987</v>
       </c>
       <c r="W11" t="n">
-        <v>9.6211</v>
+        <v>0</v>
       </c>
       <c r="X11" t="n">
-        <v>-5.1846</v>
+        <v>-3.6987</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>J. MARCOS</t>
+          <t>W. HERNANGOMEZ</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1342,76 +1342,76 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="D12" t="n">
-        <v>0.7706000000000004</v>
+        <v>-0.275</v>
       </c>
       <c r="E12" t="n">
-        <v>-4.9995</v>
+        <v>-0.1918</v>
       </c>
       <c r="F12" t="n">
-        <v>5.7704</v>
+        <v>-0.08320000000000001</v>
       </c>
       <c r="G12" t="n">
-        <v>9.9842</v>
+        <v>-0.6063999999999999</v>
       </c>
       <c r="H12" t="n">
-        <v>6.1067</v>
+        <v>-1.3847</v>
       </c>
       <c r="I12" t="n">
-        <v>3.877200000000001</v>
+        <v>0.7782</v>
       </c>
       <c r="J12" t="n">
-        <v>11.8903</v>
+        <v>-0.862</v>
       </c>
       <c r="K12" t="n">
-        <v>3.1409</v>
+        <v>-0.9732000000000001</v>
       </c>
       <c r="L12" t="n">
-        <v>8.749599999999999</v>
+        <v>0.1112</v>
       </c>
       <c r="M12" t="n">
-        <v>-1.9067</v>
+        <v>0.2555</v>
       </c>
       <c r="N12" t="n">
-        <v>2.9661</v>
+        <v>-0.4115</v>
       </c>
       <c r="O12" t="n">
-        <v>-4.8728</v>
+        <v>0.667</v>
       </c>
       <c r="P12" t="n">
-        <v>-4.8966</v>
+        <v>0.6885</v>
       </c>
       <c r="Q12" t="n">
-        <v>-15.156</v>
+        <v>0</v>
       </c>
       <c r="R12" t="n">
-        <v>10.2594</v>
+        <v>0.6885</v>
       </c>
       <c r="S12" t="n">
-        <v>1.2493</v>
+        <v>0.7249</v>
       </c>
       <c r="T12" t="n">
-        <v>-1.7341</v>
+        <v>0.6703</v>
       </c>
       <c r="U12" t="n">
-        <v>2.983</v>
+        <v>0.05479999999999996</v>
       </c>
       <c r="V12" t="n">
-        <v>-5.5657</v>
+        <v>-1.082</v>
       </c>
       <c r="W12" t="n">
         <v>0</v>
       </c>
       <c r="X12" t="n">
-        <v>-5.5657</v>
+        <v>-1.082</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>W. HERNANGOMEZ</t>
+          <t>K. PUNTER</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1420,70 +1420,70 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D13" t="n">
-        <v>-1.5241</v>
+        <v>-2.5678</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.6511</v>
+        <v>-4.3195</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.8729999999999999</v>
+        <v>1.7515</v>
       </c>
       <c r="G13" t="n">
-        <v>-2.4572</v>
+        <v>-3.9306</v>
       </c>
       <c r="H13" t="n">
-        <v>-3.6083</v>
+        <v>-2.9504</v>
       </c>
       <c r="I13" t="n">
-        <v>1.1511</v>
+        <v>-0.9802000000000004</v>
       </c>
       <c r="J13" t="n">
-        <v>-1.6052</v>
+        <v>-2.6738</v>
       </c>
       <c r="K13" t="n">
-        <v>-1.7887</v>
+        <v>-2.9124</v>
       </c>
       <c r="L13" t="n">
-        <v>0.1835</v>
+        <v>0.2385999999999999</v>
       </c>
       <c r="M13" t="n">
-        <v>-0.8519</v>
+        <v>-1.2569</v>
       </c>
       <c r="N13" t="n">
-        <v>-1.8199</v>
+        <v>-0.03809999999999991</v>
       </c>
       <c r="O13" t="n">
-        <v>0.9676</v>
+        <v>-1.2188</v>
       </c>
       <c r="P13" t="n">
-        <v>0.6995</v>
+        <v>0.6884999999999999</v>
       </c>
       <c r="Q13" t="n">
-        <v>0</v>
+        <v>-3.9015</v>
       </c>
       <c r="R13" t="n">
-        <v>0.6995</v>
+        <v>4.59</v>
       </c>
       <c r="S13" t="n">
-        <v>2.1247</v>
+        <v>0.7368</v>
       </c>
       <c r="T13" t="n">
-        <v>0.9542</v>
+        <v>-0.2099</v>
       </c>
       <c r="U13" t="n">
-        <v>1.1708</v>
+        <v>0.9465999999999999</v>
       </c>
       <c r="V13" t="n">
-        <v>-1.8911</v>
+        <v>-0.06239999999999979</v>
       </c>
       <c r="W13" t="n">
-        <v>0</v>
+        <v>2.4658</v>
       </c>
       <c r="X13" t="n">
-        <v>-1.8911</v>
+        <v>-2.5282</v>
       </c>
     </row>
     <row r="14">
@@ -1498,70 +1498,70 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="D14" t="n">
-        <v>191.645</v>
+        <v>83.04709999999999</v>
       </c>
       <c r="E14" t="n">
-        <v>95.17490000000001</v>
+        <v>29.4824</v>
       </c>
       <c r="F14" t="n">
-        <v>96.46899999999999</v>
+        <v>53.56440000000001</v>
       </c>
       <c r="G14" t="n">
-        <v>151.1125</v>
+        <v>72.8965</v>
       </c>
       <c r="H14" t="n">
-        <v>43.3006</v>
+        <v>22.0334</v>
       </c>
       <c r="I14" t="n">
-        <v>107.8134</v>
+        <v>50.8632</v>
       </c>
       <c r="J14" t="n">
-        <v>156.7391</v>
+        <v>58.13609999999999</v>
       </c>
       <c r="K14" t="n">
-        <v>48.57319999999999</v>
+        <v>15.3291</v>
       </c>
       <c r="L14" t="n">
-        <v>108.1664</v>
+        <v>42.8075</v>
       </c>
       <c r="M14" t="n">
-        <v>-5.627300000000001</v>
+        <v>14.7603</v>
       </c>
       <c r="N14" t="n">
-        <v>-5.273099999999999</v>
+        <v>6.704499999999999</v>
       </c>
       <c r="O14" t="n">
-        <v>-0.3539000000000021</v>
+        <v>8.056099999999999</v>
       </c>
       <c r="P14" t="n">
-        <v>-10.4926</v>
+        <v>-4.589799999999999</v>
       </c>
       <c r="Q14" t="n">
-        <v>-146.895</v>
+        <v>-53.932</v>
       </c>
       <c r="R14" t="n">
-        <v>136.4023</v>
+        <v>49.34249999999999</v>
       </c>
       <c r="S14" t="n">
-        <v>30.9137</v>
+        <v>10.9273</v>
       </c>
       <c r="T14" t="n">
-        <v>-3.686</v>
+        <v>-3.4943</v>
       </c>
       <c r="U14" t="n">
-        <v>34.5992</v>
+        <v>14.4216</v>
       </c>
       <c r="V14" t="n">
-        <v>20.1108</v>
+        <v>3.812799999999999</v>
       </c>
       <c r="W14" t="n">
-        <v>89.01690000000001</v>
+        <v>28.7723</v>
       </c>
       <c r="X14" t="n">
-        <v>-68.90609999999998</v>
+        <v>-24.9593</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
new cor 3 fix EL_ new game ACB
</commit_message>
<xml_diff>
--- a/informes_data/ACB/2025-26/playoffs/aggregate_individual/AGG_IND_Barça.xlsx
+++ b/informes_data/ACB/2025-26/playoffs/aggregate_individual/AGG_IND_Barça.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X14"/>
+  <dimension ref="A1:X15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -553,7 +553,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>D. BRIZUELA</t>
+          <t>J. PARRA</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -562,76 +562,76 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D2" t="n">
-        <v>18.3027</v>
+        <v>22.0422</v>
       </c>
       <c r="E2" t="n">
-        <v>8.220800000000001</v>
+        <v>15.8347</v>
       </c>
       <c r="F2" t="n">
-        <v>10.082</v>
+        <v>6.2077</v>
       </c>
       <c r="G2" t="n">
-        <v>13.6491</v>
+        <v>18.3166</v>
       </c>
       <c r="H2" t="n">
-        <v>9.77</v>
+        <v>2.7831</v>
       </c>
       <c r="I2" t="n">
-        <v>3.8793</v>
+        <v>15.5334</v>
       </c>
       <c r="J2" t="n">
-        <v>10.3187</v>
+        <v>16.5535</v>
       </c>
       <c r="K2" t="n">
-        <v>9.289199999999999</v>
+        <v>4.5419</v>
       </c>
       <c r="L2" t="n">
-        <v>1.0298</v>
+        <v>12.0116</v>
       </c>
       <c r="M2" t="n">
-        <v>3.3303</v>
+        <v>1.762900000000001</v>
       </c>
       <c r="N2" t="n">
-        <v>0.4808999999999999</v>
+        <v>-1.7589</v>
       </c>
       <c r="O2" t="n">
-        <v>2.8494</v>
+        <v>3.5219</v>
       </c>
       <c r="P2" t="n">
-        <v>1.6244</v>
+        <v>7.0129</v>
       </c>
       <c r="Q2" t="n">
-        <v>-5.8018</v>
+        <v>-2.5714</v>
       </c>
       <c r="R2" t="n">
-        <v>7.4263</v>
+        <v>9.584300000000001</v>
       </c>
       <c r="S2" t="n">
-        <v>1.8159</v>
+        <v>-1.0223</v>
       </c>
       <c r="T2" t="n">
-        <v>0.2059000000000001</v>
+        <v>-0.8098000000000001</v>
       </c>
       <c r="U2" t="n">
-        <v>1.6101</v>
+        <v>-0.2125</v>
       </c>
       <c r="V2" t="n">
-        <v>1.2131</v>
+        <v>-2.265</v>
       </c>
       <c r="W2" t="n">
-        <v>3.4978</v>
+        <v>2.6623</v>
       </c>
       <c r="X2" t="n">
-        <v>-2.2848</v>
+        <v>-4.9273</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>J. PARRA</t>
+          <t>D. BRIZUELA</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -640,76 +640,76 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D3" t="n">
-        <v>16.2031</v>
+        <v>15.4</v>
       </c>
       <c r="E3" t="n">
-        <v>9.715</v>
+        <v>7.5444</v>
       </c>
       <c r="F3" t="n">
-        <v>6.4883</v>
+        <v>7.8559</v>
       </c>
       <c r="G3" t="n">
-        <v>12.8065</v>
+        <v>13.4763</v>
       </c>
       <c r="H3" t="n">
-        <v>2.6927</v>
+        <v>8.0595</v>
       </c>
       <c r="I3" t="n">
-        <v>10.1137</v>
+        <v>5.4169</v>
       </c>
       <c r="J3" t="n">
-        <v>10.4432</v>
+        <v>10.3327</v>
       </c>
       <c r="K3" t="n">
-        <v>3.1352</v>
+        <v>7.6306</v>
       </c>
       <c r="L3" t="n">
-        <v>7.307799999999999</v>
+        <v>2.7021</v>
       </c>
       <c r="M3" t="n">
-        <v>2.363200000000001</v>
+        <v>3.1435</v>
       </c>
       <c r="N3" t="n">
-        <v>-0.4425</v>
+        <v>0.4289999999999999</v>
       </c>
       <c r="O3" t="n">
-        <v>2.8057</v>
+        <v>2.7147</v>
       </c>
       <c r="P3" t="n">
-        <v>6.266</v>
+        <v>1.8702</v>
       </c>
       <c r="Q3" t="n">
-        <v>-2.5529</v>
+        <v>-5.8442</v>
       </c>
       <c r="R3" t="n">
-        <v>8.8188</v>
+        <v>7.7144</v>
       </c>
       <c r="S3" t="n">
-        <v>-0.04859999999999998</v>
+        <v>0.9836</v>
       </c>
       <c r="T3" t="n">
-        <v>-0.3189000000000001</v>
+        <v>-0.4093000000000001</v>
       </c>
       <c r="U3" t="n">
-        <v>0.2703000000000001</v>
+        <v>1.3927</v>
       </c>
       <c r="V3" t="n">
-        <v>-2.8206</v>
+        <v>-0.9299000000000002</v>
       </c>
       <c r="W3" t="n">
-        <v>2.1434</v>
+        <v>3.4649</v>
       </c>
       <c r="X3" t="n">
-        <v>-4.964</v>
+        <v>-4.3949</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>J. VESELY</t>
+          <t>N. LAPROVITTOLA</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -721,73 +721,73 @@
         <v>6</v>
       </c>
       <c r="D4" t="n">
-        <v>13.3074</v>
+        <v>14.7661</v>
       </c>
       <c r="E4" t="n">
-        <v>8.6668</v>
+        <v>14.0761</v>
       </c>
       <c r="F4" t="n">
-        <v>4.6406</v>
+        <v>0.6899</v>
       </c>
       <c r="G4" t="n">
-        <v>3.7665</v>
+        <v>22.0596</v>
       </c>
       <c r="H4" t="n">
-        <v>3.3707</v>
+        <v>1.8269</v>
       </c>
       <c r="I4" t="n">
-        <v>0.3956999999999999</v>
+        <v>20.2327</v>
       </c>
       <c r="J4" t="n">
-        <v>6.3077</v>
+        <v>23.9044</v>
       </c>
       <c r="K4" t="n">
-        <v>4.5923</v>
+        <v>3.8767</v>
       </c>
       <c r="L4" t="n">
-        <v>1.7153</v>
+        <v>20.0278</v>
       </c>
       <c r="M4" t="n">
-        <v>-2.5414</v>
+        <v>-1.8449</v>
       </c>
       <c r="N4" t="n">
-        <v>-1.2217</v>
+        <v>-2.0497</v>
       </c>
       <c r="O4" t="n">
-        <v>-1.3195</v>
+        <v>0.2049000000000001</v>
       </c>
       <c r="P4" t="n">
-        <v>3.9452</v>
+        <v>-11.6882</v>
       </c>
       <c r="Q4" t="n">
-        <v>-3.9454</v>
+        <v>-17.2987</v>
       </c>
       <c r="R4" t="n">
-        <v>7.890400000000001</v>
+        <v>5.610300000000001</v>
       </c>
       <c r="S4" t="n">
-        <v>0.9439000000000001</v>
+        <v>0.9297</v>
       </c>
       <c r="T4" t="n">
-        <v>-0.4087</v>
+        <v>-0.2544999999999999</v>
       </c>
       <c r="U4" t="n">
-        <v>1.3527</v>
+        <v>1.1842</v>
       </c>
       <c r="V4" t="n">
-        <v>4.651899999999999</v>
+        <v>3.4649</v>
       </c>
       <c r="W4" t="n">
-        <v>6.712800000000001</v>
+        <v>7.724699999999999</v>
       </c>
       <c r="X4" t="n">
-        <v>-2.0612</v>
+        <v>-4.2597</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>T. SHENGELIA</t>
+          <t>J. VESELY</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -796,76 +796,76 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D5" t="n">
-        <v>11.3468</v>
+        <v>12.9582</v>
       </c>
       <c r="E5" t="n">
-        <v>9.1402</v>
+        <v>8.4628</v>
       </c>
       <c r="F5" t="n">
-        <v>2.206799999999999</v>
+        <v>4.4953</v>
       </c>
       <c r="G5" t="n">
-        <v>1.3805</v>
+        <v>3.1752</v>
       </c>
       <c r="H5" t="n">
-        <v>2.7901</v>
+        <v>0.9182000000000001</v>
       </c>
       <c r="I5" t="n">
-        <v>-1.4095</v>
+        <v>2.2568</v>
       </c>
       <c r="J5" t="n">
-        <v>5.9552</v>
+        <v>5.7413</v>
       </c>
       <c r="K5" t="n">
-        <v>4.0396</v>
+        <v>3.6545</v>
       </c>
       <c r="L5" t="n">
-        <v>1.9154</v>
+        <v>2.0867</v>
       </c>
       <c r="M5" t="n">
-        <v>-4.5745</v>
+        <v>-2.5661</v>
       </c>
       <c r="N5" t="n">
-        <v>-1.2496</v>
+        <v>-2.7362</v>
       </c>
       <c r="O5" t="n">
-        <v>-3.3249</v>
+        <v>0.1702000000000001</v>
       </c>
       <c r="P5" t="n">
-        <v>-3.249</v>
+        <v>4.6754</v>
       </c>
       <c r="Q5" t="n">
-        <v>-10.2113</v>
+        <v>-3.974</v>
       </c>
       <c r="R5" t="n">
-        <v>6.9622</v>
+        <v>8.6494</v>
       </c>
       <c r="S5" t="n">
-        <v>5.2503</v>
+        <v>1.1259</v>
       </c>
       <c r="T5" t="n">
-        <v>2.2549</v>
+        <v>-1.0291</v>
       </c>
       <c r="U5" t="n">
-        <v>2.9953</v>
+        <v>2.1549</v>
       </c>
       <c r="V5" t="n">
-        <v>7.9648</v>
+        <v>3.9819</v>
       </c>
       <c r="W5" t="n">
-        <v>11.1411</v>
+        <v>7.7247</v>
       </c>
       <c r="X5" t="n">
-        <v>-3.1763</v>
+        <v>-3.7429</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>N. LAPROVITTOLA</t>
+          <t>W. CLYBURN</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -874,76 +874,76 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D6" t="n">
-        <v>11.2478</v>
+        <v>11.1942</v>
       </c>
       <c r="E6" t="n">
-        <v>8.802600000000002</v>
+        <v>8.4823</v>
       </c>
       <c r="F6" t="n">
-        <v>2.4451</v>
+        <v>2.7121</v>
       </c>
       <c r="G6" t="n">
-        <v>14.4339</v>
+        <v>12.4153</v>
       </c>
       <c r="H6" t="n">
-        <v>1.4414</v>
+        <v>-1.2454</v>
       </c>
       <c r="I6" t="n">
-        <v>12.9923</v>
+        <v>13.6607</v>
       </c>
       <c r="J6" t="n">
-        <v>15.1162</v>
+        <v>17.0932</v>
       </c>
       <c r="K6" t="n">
-        <v>1.7491</v>
+        <v>2.670500000000001</v>
       </c>
       <c r="L6" t="n">
-        <v>13.3671</v>
+        <v>14.4226</v>
       </c>
       <c r="M6" t="n">
-        <v>-0.6821999999999999</v>
+        <v>-4.677899999999999</v>
       </c>
       <c r="N6" t="n">
-        <v>-0.3077</v>
+        <v>-3.916</v>
       </c>
       <c r="O6" t="n">
-        <v>-0.3746999999999999</v>
+        <v>-0.7618999999999999</v>
       </c>
       <c r="P6" t="n">
-        <v>-9.050799999999999</v>
+        <v>-6.078</v>
       </c>
       <c r="Q6" t="n">
-        <v>-13.4603</v>
+        <v>-16.3636</v>
       </c>
       <c r="R6" t="n">
-        <v>4.4094</v>
+        <v>10.2857</v>
       </c>
       <c r="S6" t="n">
-        <v>1.5778</v>
+        <v>3.3373</v>
       </c>
       <c r="T6" t="n">
-        <v>0.7163</v>
+        <v>0.4254</v>
       </c>
       <c r="U6" t="n">
-        <v>0.8613999999999999</v>
+        <v>2.9119</v>
       </c>
       <c r="V6" t="n">
-        <v>4.2868</v>
+        <v>1.5194</v>
       </c>
       <c r="W6" t="n">
-        <v>6.4302</v>
+        <v>7.3273</v>
       </c>
       <c r="X6" t="n">
-        <v>-2.1434</v>
+        <v>-5.807700000000001</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>W. CLYBURN</t>
+          <t>T. SHENGELIA</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -952,70 +952,70 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D7" t="n">
-        <v>10.9561</v>
+        <v>8.3553</v>
       </c>
       <c r="E7" t="n">
-        <v>7.4752</v>
+        <v>7.622300000000001</v>
       </c>
       <c r="F7" t="n">
-        <v>3.4809</v>
+        <v>0.7329999999999999</v>
       </c>
       <c r="G7" t="n">
-        <v>10.8409</v>
+        <v>1.0942</v>
       </c>
       <c r="H7" t="n">
-        <v>-1.2203</v>
+        <v>2.593</v>
       </c>
       <c r="I7" t="n">
-        <v>12.0613</v>
+        <v>-1.4987</v>
       </c>
       <c r="J7" t="n">
-        <v>14.8641</v>
+        <v>7.24</v>
       </c>
       <c r="K7" t="n">
-        <v>1.2327</v>
+        <v>5.5034</v>
       </c>
       <c r="L7" t="n">
-        <v>13.6315</v>
+        <v>1.7366</v>
       </c>
       <c r="M7" t="n">
-        <v>-4.0232</v>
+        <v>-6.145799999999999</v>
       </c>
       <c r="N7" t="n">
-        <v>-2.453</v>
+        <v>-2.9105</v>
       </c>
       <c r="O7" t="n">
-        <v>-1.5702</v>
+        <v>-3.2353</v>
       </c>
       <c r="P7" t="n">
-        <v>-5.1056</v>
+        <v>-5.3765</v>
       </c>
       <c r="Q7" t="n">
-        <v>-14.8526</v>
+        <v>-12.8571</v>
       </c>
       <c r="R7" t="n">
-        <v>9.747</v>
+        <v>7.4805</v>
       </c>
       <c r="S7" t="n">
-        <v>3.6861</v>
+        <v>6.056</v>
       </c>
       <c r="T7" t="n">
-        <v>0.7507</v>
+        <v>2.4473</v>
       </c>
       <c r="U7" t="n">
-        <v>2.9355</v>
+        <v>3.6086</v>
       </c>
       <c r="V7" t="n">
-        <v>1.5346</v>
+        <v>6.581799999999999</v>
       </c>
       <c r="W7" t="n">
-        <v>6.7129</v>
+        <v>10.7923</v>
       </c>
       <c r="X7" t="n">
-        <v>-5.1783</v>
+        <v>-4.2104</v>
       </c>
     </row>
     <row r="8">
@@ -1030,70 +1030,70 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D8" t="n">
-        <v>8.3283</v>
+        <v>7.6255</v>
       </c>
       <c r="E8" t="n">
-        <v>6.6893</v>
+        <v>5.1698</v>
       </c>
       <c r="F8" t="n">
-        <v>1.6389</v>
+        <v>2.4556</v>
       </c>
       <c r="G8" t="n">
-        <v>5.0835</v>
+        <v>5.0234</v>
       </c>
       <c r="H8" t="n">
-        <v>5.3523</v>
+        <v>5.5136</v>
       </c>
       <c r="I8" t="n">
-        <v>-0.2687</v>
+        <v>-0.4902</v>
       </c>
       <c r="J8" t="n">
-        <v>6.3893</v>
+        <v>6.322</v>
       </c>
       <c r="K8" t="n">
-        <v>5.5432</v>
+        <v>5.4064</v>
       </c>
       <c r="L8" t="n">
-        <v>0.8464</v>
+        <v>0.9155</v>
       </c>
       <c r="M8" t="n">
-        <v>-1.3058</v>
+        <v>-1.2988</v>
       </c>
       <c r="N8" t="n">
-        <v>-0.1907</v>
+        <v>0.1072</v>
       </c>
       <c r="O8" t="n">
-        <v>-1.1151</v>
+        <v>-1.406</v>
       </c>
       <c r="P8" t="n">
-        <v>1.3923</v>
+        <v>0.4675</v>
       </c>
       <c r="Q8" t="n">
-        <v>-3.0171</v>
+        <v>-4.4416</v>
       </c>
       <c r="R8" t="n">
-        <v>4.4093</v>
+        <v>4.909000000000001</v>
       </c>
       <c r="S8" t="n">
-        <v>4.322</v>
+        <v>5.3995</v>
       </c>
       <c r="T8" t="n">
-        <v>1.6799</v>
+        <v>2.4789</v>
       </c>
       <c r="U8" t="n">
-        <v>2.6421</v>
+        <v>2.9205</v>
       </c>
       <c r="V8" t="n">
-        <v>-2.4696</v>
+        <v>-3.265</v>
       </c>
       <c r="W8" t="n">
-        <v>1.6371</v>
+        <v>0.8103</v>
       </c>
       <c r="X8" t="n">
-        <v>-4.1067</v>
+        <v>-4.0753</v>
       </c>
     </row>
     <row r="9">
@@ -1111,73 +1111,73 @@
         <v>6</v>
       </c>
       <c r="D9" t="n">
-        <v>6.728999999999999</v>
+        <v>6.7961</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.6759999999999998</v>
+        <v>-0.9267000000000001</v>
       </c>
       <c r="F9" t="n">
-        <v>7.4051</v>
+        <v>7.7229</v>
       </c>
       <c r="G9" t="n">
-        <v>6.8101</v>
+        <v>6.8956</v>
       </c>
       <c r="H9" t="n">
-        <v>-1.5972</v>
+        <v>-1.568</v>
       </c>
       <c r="I9" t="n">
-        <v>8.407400000000001</v>
+        <v>8.4636</v>
       </c>
       <c r="J9" t="n">
-        <v>5.6333</v>
+        <v>5.4412</v>
       </c>
       <c r="K9" t="n">
-        <v>-0.04890000000000017</v>
+        <v>-0.1791999999999998</v>
       </c>
       <c r="L9" t="n">
-        <v>5.682</v>
+        <v>5.6204</v>
       </c>
       <c r="M9" t="n">
-        <v>1.1771</v>
+        <v>1.4542</v>
       </c>
       <c r="N9" t="n">
-        <v>-1.5483</v>
+        <v>-1.389</v>
       </c>
       <c r="O9" t="n">
-        <v>2.7254</v>
+        <v>2.8431</v>
       </c>
       <c r="P9" t="n">
-        <v>0.000100000000000211</v>
+        <v>-9.999999999976694e-05</v>
       </c>
       <c r="Q9" t="n">
-        <v>-7.6584</v>
+        <v>-7.7143</v>
       </c>
       <c r="R9" t="n">
-        <v>7.6584</v>
+        <v>7.7142</v>
       </c>
       <c r="S9" t="n">
-        <v>-0.2227</v>
+        <v>-0.2344</v>
       </c>
       <c r="T9" t="n">
-        <v>-1.0769</v>
+        <v>-1.0536</v>
       </c>
       <c r="U9" t="n">
-        <v>0.8545</v>
+        <v>0.8193999999999999</v>
       </c>
       <c r="V9" t="n">
-        <v>0.1413</v>
+        <v>0.1351</v>
       </c>
       <c r="W9" t="n">
-        <v>2.426</v>
+        <v>2.4</v>
       </c>
       <c r="X9" t="n">
-        <v>-2.2847</v>
+        <v>-2.2649</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>W. HERNANGOMEZ</t>
+          <t>M. CALE</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1186,76 +1186,76 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D10" t="n">
-        <v>3.6795</v>
+        <v>5.1303</v>
       </c>
       <c r="E10" t="n">
-        <v>0.9387</v>
+        <v>1.2094</v>
       </c>
       <c r="F10" t="n">
-        <v>2.7407</v>
+        <v>3.921</v>
       </c>
       <c r="G10" t="n">
-        <v>1.0268</v>
+        <v>4.4786</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.8611999999999999</v>
+        <v>0.7409999999999998</v>
       </c>
       <c r="I10" t="n">
-        <v>1.888</v>
+        <v>3.7375</v>
       </c>
       <c r="J10" t="n">
-        <v>-0.5199</v>
+        <v>3.727</v>
       </c>
       <c r="K10" t="n">
-        <v>-0.7775000000000001</v>
+        <v>1.1473</v>
       </c>
       <c r="L10" t="n">
-        <v>0.2576</v>
+        <v>2.5797</v>
       </c>
       <c r="M10" t="n">
-        <v>1.5468</v>
+        <v>0.7514999999999998</v>
       </c>
       <c r="N10" t="n">
-        <v>-0.08379999999999999</v>
+        <v>-0.4061999999999999</v>
       </c>
       <c r="O10" t="n">
-        <v>1.6305</v>
+        <v>1.1578</v>
       </c>
       <c r="P10" t="n">
-        <v>2.7848</v>
+        <v>1.4026</v>
       </c>
       <c r="Q10" t="n">
-        <v>0</v>
+        <v>-3.7402</v>
       </c>
       <c r="R10" t="n">
-        <v>2.7848</v>
+        <v>5.1429</v>
       </c>
       <c r="S10" t="n">
-        <v>1.8699</v>
+        <v>-0.4885</v>
       </c>
       <c r="T10" t="n">
-        <v>1.0347</v>
+        <v>-1.1773</v>
       </c>
       <c r="U10" t="n">
-        <v>0.8353</v>
+        <v>0.6887999999999999</v>
       </c>
       <c r="V10" t="n">
-        <v>-2.0021</v>
+        <v>-0.2624</v>
       </c>
       <c r="W10" t="n">
-        <v>0.424</v>
+        <v>2.3999</v>
       </c>
       <c r="X10" t="n">
-        <v>-2.4261</v>
+        <v>-2.6623</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>M. CALE</t>
+          <t>W. HERNANGOMEZ</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1264,70 +1264,70 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D11" t="n">
-        <v>3.3168</v>
+        <v>1.942</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.2050000000000001</v>
+        <v>0.05189999999999995</v>
       </c>
       <c r="F11" t="n">
-        <v>3.5218</v>
+        <v>1.8901</v>
       </c>
       <c r="G11" t="n">
-        <v>3.9746</v>
+        <v>-0.2208000000000001</v>
       </c>
       <c r="H11" t="n">
-        <v>1.4865</v>
+        <v>-2.0538</v>
       </c>
       <c r="I11" t="n">
-        <v>2.4882</v>
+        <v>1.8329</v>
       </c>
       <c r="J11" t="n">
-        <v>2.7191</v>
+        <v>-1.3257</v>
       </c>
       <c r="K11" t="n">
-        <v>1.2015</v>
+        <v>-1.6918</v>
       </c>
       <c r="L11" t="n">
-        <v>1.5176</v>
+        <v>0.3662</v>
       </c>
       <c r="M11" t="n">
-        <v>1.2557</v>
+        <v>1.1048</v>
       </c>
       <c r="N11" t="n">
-        <v>0.2851000000000001</v>
+        <v>-0.3619</v>
       </c>
       <c r="O11" t="n">
-        <v>0.9705000000000001</v>
+        <v>1.4667</v>
       </c>
       <c r="P11" t="n">
-        <v>0.9283</v>
+        <v>2.8052</v>
       </c>
       <c r="Q11" t="n">
-        <v>-3.7133</v>
+        <v>0</v>
       </c>
       <c r="R11" t="n">
-        <v>4.641500000000001</v>
+        <v>2.8052</v>
       </c>
       <c r="S11" t="n">
-        <v>-0.2611</v>
+        <v>1.3524</v>
       </c>
       <c r="T11" t="n">
-        <v>-0.5650999999999999</v>
+        <v>0.9723000000000001</v>
       </c>
       <c r="U11" t="n">
-        <v>0.3041</v>
+        <v>0.3802</v>
       </c>
       <c r="V11" t="n">
-        <v>-1.3249</v>
+        <v>-1.9947</v>
       </c>
       <c r="W11" t="n">
-        <v>1.3544</v>
+        <v>0.4052</v>
       </c>
       <c r="X11" t="n">
-        <v>-2.6793</v>
+        <v>-2.3999</v>
       </c>
     </row>
     <row r="12">
@@ -1342,76 +1342,76 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D12" t="n">
-        <v>0.2843000000000002</v>
+        <v>0.4275</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.9266000000000002</v>
+        <v>-1.5502</v>
       </c>
       <c r="F12" t="n">
-        <v>1.2107</v>
+        <v>1.9777</v>
       </c>
       <c r="G12" t="n">
-        <v>3.067</v>
+        <v>3.4577</v>
       </c>
       <c r="H12" t="n">
-        <v>2.3746</v>
+        <v>1.7537</v>
       </c>
       <c r="I12" t="n">
-        <v>0.6922999999999999</v>
+        <v>1.7038</v>
       </c>
       <c r="J12" t="n">
-        <v>5.8743</v>
+        <v>6.4472</v>
       </c>
       <c r="K12" t="n">
-        <v>2.2295</v>
+        <v>1.9816</v>
       </c>
       <c r="L12" t="n">
-        <v>3.6446</v>
+        <v>4.4655</v>
       </c>
       <c r="M12" t="n">
-        <v>-2.8073</v>
+        <v>-2.9894</v>
       </c>
       <c r="N12" t="n">
-        <v>0.1451</v>
+        <v>-0.2279</v>
       </c>
       <c r="O12" t="n">
-        <v>-2.9524</v>
+        <v>-2.7615</v>
       </c>
       <c r="P12" t="n">
-        <v>-1.1604</v>
+        <v>-2.3377</v>
       </c>
       <c r="Q12" t="n">
-        <v>-5.8018</v>
+        <v>-7.0129</v>
       </c>
       <c r="R12" t="n">
-        <v>4.6413</v>
+        <v>4.6753</v>
       </c>
       <c r="S12" t="n">
-        <v>0.4822</v>
+        <v>0.7282000000000001</v>
       </c>
       <c r="T12" t="n">
-        <v>-0.9989999999999999</v>
+        <v>-0.9843</v>
       </c>
       <c r="U12" t="n">
-        <v>1.4813</v>
+        <v>1.7125</v>
       </c>
       <c r="V12" t="n">
-        <v>-2.1045</v>
+        <v>-1.4209</v>
       </c>
       <c r="W12" t="n">
         <v>0</v>
       </c>
       <c r="X12" t="n">
-        <v>-2.1045</v>
+        <v>-1.4209</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>K. PUNTER</t>
+          <t>J. NUNEZ</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1420,148 +1420,226 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.6343999999999999</v>
+        <v>-0.3094</v>
       </c>
       <c r="E13" t="n">
-        <v>1.6166</v>
+        <v>0.5854</v>
       </c>
       <c r="F13" t="n">
-        <v>-2.251</v>
+        <v>-0.8948</v>
       </c>
       <c r="G13" t="n">
-        <v>1.664099999999999</v>
+        <v>-0.1033</v>
       </c>
       <c r="H13" t="n">
-        <v>-2.229</v>
+        <v>-0.5612</v>
       </c>
       <c r="I13" t="n">
-        <v>3.8931</v>
+        <v>0.4579</v>
       </c>
       <c r="J13" t="n">
-        <v>6.974699999999999</v>
+        <v>0.5994</v>
       </c>
       <c r="K13" t="n">
-        <v>-0.4478999999999997</v>
+        <v>-0.0598</v>
       </c>
       <c r="L13" t="n">
-        <v>7.4227</v>
+        <v>0.6592</v>
       </c>
       <c r="M13" t="n">
-        <v>-5.3109</v>
+        <v>-0.7027</v>
       </c>
       <c r="N13" t="n">
-        <v>-1.7813</v>
+        <v>-0.5014</v>
       </c>
       <c r="O13" t="n">
-        <v>-3.5295</v>
+        <v>-0.2013</v>
       </c>
       <c r="P13" t="n">
-        <v>-4.1774</v>
+        <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v>-10.2112</v>
+        <v>0</v>
       </c>
       <c r="R13" t="n">
-        <v>6.0339</v>
+        <v>0</v>
       </c>
       <c r="S13" t="n">
-        <v>0.2324999999999999</v>
+        <v>-0.2061</v>
       </c>
       <c r="T13" t="n">
-        <v>-0.2523</v>
+        <v>-0.0141</v>
       </c>
       <c r="U13" t="n">
-        <v>0.4850000000000001</v>
+        <v>-0.192</v>
       </c>
       <c r="V13" t="n">
-        <v>1.6464</v>
+        <v>0</v>
       </c>
       <c r="W13" t="n">
-        <v>5.105300000000001</v>
+        <v>0</v>
       </c>
       <c r="X13" t="n">
-        <v>-3.459</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>K. PUNTER</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Barça</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>7</v>
+      </c>
+      <c r="D14" t="n">
+        <v>-2.5738</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1.0629</v>
+      </c>
+      <c r="F14" t="n">
+        <v>-3.6365</v>
+      </c>
+      <c r="G14" t="n">
+        <v>1.3815</v>
+      </c>
+      <c r="H14" t="n">
+        <v>-4.6979</v>
+      </c>
+      <c r="I14" t="n">
+        <v>6.0796</v>
+      </c>
+      <c r="J14" t="n">
+        <v>8.3691</v>
+      </c>
+      <c r="K14" t="n">
+        <v>-0.4508</v>
+      </c>
+      <c r="L14" t="n">
+        <v>8.8201</v>
+      </c>
+      <c r="M14" t="n">
+        <v>-6.9876</v>
+      </c>
+      <c r="N14" t="n">
+        <v>-4.2471</v>
+      </c>
+      <c r="O14" t="n">
+        <v>-2.7407</v>
+      </c>
+      <c r="P14" t="n">
+        <v>-5.6104</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>-12.8571</v>
+      </c>
+      <c r="R14" t="n">
+        <v>7.2468</v>
+      </c>
+      <c r="S14" t="n">
+        <v>0.008299999999999974</v>
+      </c>
+      <c r="T14" t="n">
+        <v>-0.5766</v>
+      </c>
+      <c r="U14" t="n">
+        <v>0.5847999999999998</v>
+      </c>
+      <c r="V14" t="n">
+        <v>1.6467</v>
+      </c>
+      <c r="W14" t="n">
+        <v>6.1271</v>
+      </c>
+      <c r="X14" t="n">
+        <v>-4.4806</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>--- TOTAL ---</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>Barça</t>
         </is>
       </c>
-      <c r="C14" t="n">
-        <v>6</v>
-      </c>
-      <c r="D14" t="n">
-        <v>103.0674</v>
-      </c>
-      <c r="E14" t="n">
-        <v>59.4576</v>
-      </c>
-      <c r="F14" t="n">
-        <v>43.6099</v>
-      </c>
-      <c r="G14" t="n">
-        <v>78.50349999999999</v>
-      </c>
-      <c r="H14" t="n">
-        <v>23.3706</v>
-      </c>
-      <c r="I14" t="n">
-        <v>55.1331</v>
-      </c>
-      <c r="J14" t="n">
-        <v>90.07589999999999</v>
-      </c>
-      <c r="K14" t="n">
-        <v>31.738</v>
-      </c>
-      <c r="L14" t="n">
-        <v>58.33779999999999</v>
-      </c>
-      <c r="M14" t="n">
-        <v>-11.5722</v>
-      </c>
-      <c r="N14" t="n">
-        <v>-8.3675</v>
-      </c>
-      <c r="O14" t="n">
-        <v>-3.204800000000001</v>
-      </c>
-      <c r="P14" t="n">
-        <v>-5.802099999999998</v>
-      </c>
-      <c r="Q14" t="n">
-        <v>-81.2261</v>
-      </c>
-      <c r="R14" t="n">
-        <v>75.4233</v>
-      </c>
-      <c r="S14" t="n">
-        <v>19.6482</v>
-      </c>
-      <c r="T14" t="n">
-        <v>3.021500000000001</v>
-      </c>
-      <c r="U14" t="n">
-        <v>16.6276</v>
-      </c>
-      <c r="V14" t="n">
-        <v>10.7172</v>
-      </c>
-      <c r="W14" t="n">
-        <v>47.585</v>
-      </c>
-      <c r="X14" t="n">
-        <v>-36.8683</v>
+      <c r="C15" t="n">
+        <v>7</v>
+      </c>
+      <c r="D15" t="n">
+        <v>103.7542</v>
+      </c>
+      <c r="E15" t="n">
+        <v>67.62510000000002</v>
+      </c>
+      <c r="F15" t="n">
+        <v>36.12989999999999</v>
+      </c>
+      <c r="G15" t="n">
+        <v>91.4499</v>
+      </c>
+      <c r="H15" t="n">
+        <v>14.0627</v>
+      </c>
+      <c r="I15" t="n">
+        <v>77.38689999999998</v>
+      </c>
+      <c r="J15" t="n">
+        <v>110.4453</v>
+      </c>
+      <c r="K15" t="n">
+        <v>34.03129999999999</v>
+      </c>
+      <c r="L15" t="n">
+        <v>76.414</v>
+      </c>
+      <c r="M15" t="n">
+        <v>-18.9963</v>
+      </c>
+      <c r="N15" t="n">
+        <v>-19.9686</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0.9726000000000004</v>
+      </c>
+      <c r="P15" t="n">
+        <v>-12.8571</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>-94.6751</v>
+      </c>
+      <c r="R15" t="n">
+        <v>81.81800000000001</v>
+      </c>
+      <c r="S15" t="n">
+        <v>17.9696</v>
+      </c>
+      <c r="T15" t="n">
+        <v>0.01530000000000054</v>
+      </c>
+      <c r="U15" t="n">
+        <v>17.954</v>
+      </c>
+      <c r="V15" t="n">
+        <v>7.1919</v>
+      </c>
+      <c r="W15" t="n">
+        <v>51.8387</v>
+      </c>
+      <c r="X15" t="n">
+        <v>-44.64680000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>